<commit_message>
all good but i want to gabung result every single map for penulisan hasil setiap map
</commit_message>
<xml_diff>
--- a/Excel/Rekap/Keseluruhan_All.xlsx
+++ b/Excel/Rekap/Keseluruhan_All.xlsx
@@ -572,22 +572,22 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>0.04537362500000001</v>
+        <v>0.04495092499999999</v>
       </c>
       <c r="C2">
-        <v>0.037133475</v>
+        <v>0.03602815</v>
       </c>
       <c r="D2">
-        <v>0.03167575</v>
+        <v>0.030476075</v>
       </c>
       <c r="E2">
-        <v>0.061977075</v>
+        <v>0.06081697500000001</v>
       </c>
       <c r="F2">
-        <v>0.095404725</v>
+        <v>0.09353719999999999</v>
       </c>
       <c r="G2">
-        <v>0.05431293</v>
+        <v>0.053161865</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -595,22 +595,22 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>0.006423900000000001</v>
+        <v>0.0064005</v>
       </c>
       <c r="C3">
-        <v>0.006966475</v>
+        <v>0.006771325000000001</v>
       </c>
       <c r="D3">
-        <v>0.005986050000000001</v>
+        <v>0.005526025</v>
       </c>
       <c r="E3">
-        <v>0.006828949999999999</v>
+        <v>0.006659575</v>
       </c>
       <c r="F3">
-        <v>0.0052471</v>
+        <v>0.005015</v>
       </c>
       <c r="G3">
-        <v>0.006290495</v>
+        <v>0.006074485</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -618,22 +618,22 @@
         <v>9</v>
       </c>
       <c r="B4">
-        <v>0.010066</v>
+        <v>0.010092325</v>
       </c>
       <c r="C4">
-        <v>0.0503714</v>
+        <v>0.04809945</v>
       </c>
       <c r="D4">
-        <v>0.01890995</v>
+        <v>0.01806635</v>
       </c>
       <c r="E4">
-        <v>0.010793</v>
+        <v>0.01053475</v>
       </c>
       <c r="F4">
-        <v>0.0072778</v>
+        <v>0.007082100000000001</v>
       </c>
       <c r="G4">
-        <v>0.01948363</v>
+        <v>0.018774995</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -641,22 +641,22 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>0.024656</v>
+        <v>0.02438905</v>
       </c>
       <c r="C5">
-        <v>0.03220025</v>
+        <v>0.0309793</v>
       </c>
       <c r="D5">
-        <v>0.0253811</v>
+        <v>0.024755975</v>
       </c>
       <c r="E5">
-        <v>0.034898075</v>
+        <v>0.03457350000000001</v>
       </c>
       <c r="F5">
-        <v>0.0454917</v>
+        <v>0.0451429</v>
       </c>
       <c r="G5">
-        <v>0.032525425</v>
+        <v>0.031968145</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -664,22 +664,22 @@
         <v>11</v>
       </c>
       <c r="B6">
-        <v>0.004847725</v>
+        <v>0.004798149999999999</v>
       </c>
       <c r="C6">
-        <v>0.004273275</v>
+        <v>0.00416185</v>
       </c>
       <c r="D6">
-        <v>0.006875825</v>
+        <v>0.00666415</v>
       </c>
       <c r="E6">
-        <v>0.006618525</v>
+        <v>0.00643215</v>
       </c>
       <c r="F6">
-        <v>0.01032265</v>
+        <v>0.010466575</v>
       </c>
       <c r="G6">
-        <v>0.006587599999999999</v>
+        <v>0.006504575</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -687,22 +687,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>0.04566025</v>
+        <v>0.04513039999999999</v>
       </c>
       <c r="C7">
-        <v>0.0375998</v>
+        <v>0.03603435</v>
       </c>
       <c r="D7">
-        <v>0.032013325</v>
+        <v>0.0311252</v>
       </c>
       <c r="E7">
-        <v>0.06195417500000001</v>
+        <v>0.06070265000000001</v>
       </c>
       <c r="F7">
-        <v>0.09722252499999999</v>
+        <v>0.09391085000000002</v>
       </c>
       <c r="G7">
-        <v>0.054890015</v>
+        <v>0.05338069000000001</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -710,22 +710,22 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>0.04300682500000001</v>
+        <v>0.04238987499999999</v>
       </c>
       <c r="C8">
-        <v>0.0354778</v>
+        <v>0.034142625</v>
       </c>
       <c r="D8">
-        <v>0.0285224</v>
+        <v>0.02728855</v>
       </c>
       <c r="E8">
-        <v>0.05846377500000001</v>
+        <v>0.05698795</v>
       </c>
       <c r="F8">
-        <v>0.09661275</v>
+        <v>0.09399302499999999</v>
       </c>
       <c r="G8">
-        <v>0.05241671000000001</v>
+        <v>0.050960405</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -733,22 +733,22 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>0.004887424999999999</v>
+        <v>0.004872</v>
       </c>
       <c r="C9">
-        <v>0.015940075</v>
+        <v>0.0155931</v>
       </c>
       <c r="D9">
-        <v>0.0069278</v>
+        <v>0.006664775</v>
       </c>
       <c r="E9">
-        <v>0.004259374999999999</v>
+        <v>0.004209424999999999</v>
       </c>
       <c r="F9">
-        <v>0.00279665</v>
+        <v>0.002743275</v>
       </c>
       <c r="G9">
-        <v>0.006962264999999998</v>
+        <v>0.006816515</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -756,22 +756,22 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>0.007675325</v>
+        <v>0.007476375</v>
       </c>
       <c r="C10">
-        <v>0.008307825000000001</v>
+        <v>0.00807475</v>
       </c>
       <c r="D10">
-        <v>0.0055774</v>
+        <v>0.005321375</v>
       </c>
       <c r="E10">
-        <v>0.0086091</v>
+        <v>0.0082272</v>
       </c>
       <c r="F10">
-        <v>0.0069488</v>
+        <v>0.00680565</v>
       </c>
       <c r="G10">
-        <v>0.007423689999999999</v>
+        <v>0.00718107</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -779,22 +779,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>0.006823099999999999</v>
+        <v>0.006691325000000001</v>
       </c>
       <c r="C11">
-        <v>0.00720205</v>
+        <v>0.007218599999999999</v>
       </c>
       <c r="D11">
-        <v>0.005979199999999999</v>
+        <v>0.005733975000000001</v>
       </c>
       <c r="E11">
-        <v>0.007173000000000001</v>
+        <v>0.0069365</v>
       </c>
       <c r="F11">
-        <v>0.0053904</v>
+        <v>0.005447550000000001</v>
       </c>
       <c r="G11">
-        <v>0.00651355</v>
+        <v>0.006405590000000001</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -802,22 +802,22 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>0.006982975000000001</v>
+        <v>0.0068519</v>
       </c>
       <c r="C12">
-        <v>0.007395325</v>
+        <v>0.00731425</v>
       </c>
       <c r="D12">
-        <v>0.0060631</v>
+        <v>0.005854974999999999</v>
       </c>
       <c r="E12">
-        <v>0.007297175</v>
+        <v>0.007199375</v>
       </c>
       <c r="F12">
-        <v>0.0053441</v>
+        <v>0.005277825</v>
       </c>
       <c r="G12">
-        <v>0.006616535</v>
+        <v>0.006499664999999999</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -825,22 +825,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>0.010447475</v>
+        <v>0.01045155</v>
       </c>
       <c r="C13">
-        <v>0.05058235</v>
+        <v>0.0488622</v>
       </c>
       <c r="D13">
-        <v>0.019190325</v>
+        <v>0.018292175</v>
       </c>
       <c r="E13">
-        <v>0.010871025</v>
+        <v>0.010616075</v>
       </c>
       <c r="F13">
-        <v>0.007564824999999999</v>
+        <v>0.0075686</v>
       </c>
       <c r="G13">
-        <v>0.0197312</v>
+        <v>0.01915812</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -848,22 +848,22 @@
         <v>19</v>
       </c>
       <c r="B14">
-        <v>0.01020105</v>
+        <v>0.010367975</v>
       </c>
       <c r="C14">
-        <v>0.04782270000000001</v>
+        <v>0.04596152499999999</v>
       </c>
       <c r="D14">
-        <v>0.0266651</v>
+        <v>0.02551215</v>
       </c>
       <c r="E14">
-        <v>0.009545350000000001</v>
+        <v>0.009463525</v>
       </c>
       <c r="F14">
-        <v>0.007026425</v>
+        <v>0.0069345</v>
       </c>
       <c r="G14">
-        <v>0.020252125</v>
+        <v>0.019647935</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -871,22 +871,22 @@
         <v>20</v>
       </c>
       <c r="B15">
-        <v>0.0160334</v>
+        <v>0.01607695</v>
       </c>
       <c r="C15">
-        <v>0.05988284999999999</v>
+        <v>0.057900125</v>
       </c>
       <c r="D15">
-        <v>0.02010065</v>
+        <v>0.018933275</v>
       </c>
       <c r="E15">
-        <v>0.009468850000000001</v>
+        <v>0.00919625</v>
       </c>
       <c r="F15">
-        <v>0.01987045</v>
+        <v>0.019279475</v>
       </c>
       <c r="G15">
-        <v>0.02507124</v>
+        <v>0.024277215</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -894,22 +894,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>0.024876</v>
+        <v>0.02475495</v>
       </c>
       <c r="C16">
-        <v>0.0325584</v>
+        <v>0.03132025</v>
       </c>
       <c r="D16">
-        <v>0.0258621</v>
+        <v>0.02525645</v>
       </c>
       <c r="E16">
-        <v>0.035321925</v>
+        <v>0.0349613</v>
       </c>
       <c r="F16">
-        <v>0.04607307499999999</v>
+        <v>0.04502727499999999</v>
       </c>
       <c r="G16">
-        <v>0.0329383</v>
+        <v>0.032264045</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -917,22 +917,22 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>0.02551265</v>
+        <v>0.025203975</v>
       </c>
       <c r="C17">
-        <v>0.03133395</v>
+        <v>0.0308002</v>
       </c>
       <c r="D17">
-        <v>0.02461715</v>
+        <v>0.0234269</v>
       </c>
       <c r="E17">
-        <v>0.032812075</v>
+        <v>0.031586725</v>
       </c>
       <c r="F17">
-        <v>0.0426814</v>
+        <v>0.041456925</v>
       </c>
       <c r="G17">
-        <v>0.031391445</v>
+        <v>0.030494945</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -940,22 +940,22 @@
         <v>23</v>
       </c>
       <c r="B18">
-        <v>0.005507225</v>
+        <v>0.005503725000000001</v>
       </c>
       <c r="C18">
-        <v>0.00384005</v>
+        <v>0.003759475</v>
       </c>
       <c r="D18">
-        <v>0.005167475</v>
+        <v>0.0050537</v>
       </c>
       <c r="E18">
-        <v>0.003604375</v>
+        <v>0.003605025</v>
       </c>
       <c r="F18">
-        <v>0.007600225</v>
+        <v>0.007552425</v>
       </c>
       <c r="G18">
-        <v>0.00514387</v>
+        <v>0.00509487</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -963,22 +963,22 @@
         <v>24</v>
       </c>
       <c r="B19">
-        <v>0.002790375</v>
+        <v>0.002771075</v>
       </c>
       <c r="C19">
-        <v>0.004072375</v>
+        <v>0.004054625</v>
       </c>
       <c r="D19">
-        <v>0.002614175</v>
+        <v>0.00252845</v>
       </c>
       <c r="E19">
-        <v>0.003013025</v>
+        <v>0.002949625</v>
       </c>
       <c r="F19">
-        <v>0.0051277</v>
+        <v>0.0052891</v>
       </c>
       <c r="G19">
-        <v>0.00352353</v>
+        <v>0.003518575</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -986,22 +986,22 @@
         <v>25</v>
       </c>
       <c r="B20">
-        <v>0.004749975</v>
+        <v>0.004767850000000001</v>
       </c>
       <c r="C20">
-        <v>0.004593524999999999</v>
+        <v>0.004616574999999999</v>
       </c>
       <c r="D20">
-        <v>0.00484465</v>
+        <v>0.0047845</v>
       </c>
       <c r="E20">
-        <v>0.004857</v>
+        <v>0.0048496</v>
       </c>
       <c r="F20">
-        <v>0.008157774999999999</v>
+        <v>0.008061075000000001</v>
       </c>
       <c r="G20">
-        <v>0.005440585</v>
+        <v>0.005415919999999999</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1009,22 +1009,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>0.004941549999999999</v>
+        <v>0.00491875</v>
       </c>
       <c r="C21">
-        <v>0.004243475</v>
+        <v>0.00424915</v>
       </c>
       <c r="D21">
-        <v>0.00681695</v>
+        <v>0.006713525000000001</v>
       </c>
       <c r="E21">
-        <v>0.0067182</v>
+        <v>0.00655855</v>
       </c>
       <c r="F21">
-        <v>0.010316725</v>
+        <v>0.01061885</v>
       </c>
       <c r="G21">
-        <v>0.00660738</v>
+        <v>0.006611765</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1032,22 +1032,22 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>0.04338085</v>
+        <v>0.04303274999999999</v>
       </c>
       <c r="C22">
-        <v>0.03585585</v>
+        <v>0.034634825</v>
       </c>
       <c r="D22">
-        <v>0.028797025</v>
+        <v>0.027536425</v>
       </c>
       <c r="E22">
-        <v>0.05846927499999999</v>
+        <v>0.05727599999999999</v>
       </c>
       <c r="F22">
-        <v>0.09736060000000001</v>
+        <v>0.09369627500000001</v>
       </c>
       <c r="G22">
-        <v>0.05277272</v>
+        <v>0.051235255</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1055,22 +1055,22 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>0.005288849999999999</v>
+        <v>0.0051491</v>
       </c>
       <c r="C23">
-        <v>0.016373075</v>
+        <v>0.01636485</v>
       </c>
       <c r="D23">
-        <v>0.007172825000000001</v>
+        <v>0.006863224999999999</v>
       </c>
       <c r="E23">
-        <v>0.0045382</v>
+        <v>0.004431450000000001</v>
       </c>
       <c r="F23">
-        <v>0.003079075</v>
+        <v>0.003000125</v>
       </c>
       <c r="G23">
-        <v>0.007290405</v>
+        <v>0.00716175</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1078,22 +1078,22 @@
         <v>29</v>
       </c>
       <c r="B24">
-        <v>0.005167275</v>
+        <v>0.0052407</v>
       </c>
       <c r="C24">
-        <v>0.01667345</v>
+        <v>0.016468875</v>
       </c>
       <c r="D24">
-        <v>0.00897835</v>
+        <v>0.00867045</v>
       </c>
       <c r="E24">
-        <v>0.004514900000000001</v>
+        <v>0.0044424</v>
       </c>
       <c r="F24">
-        <v>0.002791575</v>
+        <v>0.0027877</v>
       </c>
       <c r="G24">
-        <v>0.007625109999999999</v>
+        <v>0.007522025</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1101,22 +1101,22 @@
         <v>30</v>
       </c>
       <c r="B25">
-        <v>0.009683875</v>
+        <v>0.009783899999999998</v>
       </c>
       <c r="C25">
-        <v>0.027062275</v>
+        <v>0.02582195</v>
       </c>
       <c r="D25">
-        <v>0.01160835</v>
+        <v>0.011564225</v>
       </c>
       <c r="E25">
-        <v>0.00519125</v>
+        <v>0.005113125</v>
       </c>
       <c r="F25">
-        <v>0.01104095</v>
+        <v>0.01087075</v>
       </c>
       <c r="G25">
-        <v>0.01291734</v>
+        <v>0.01263079</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1124,22 +1124,22 @@
         <v>31</v>
       </c>
       <c r="B26">
-        <v>0.00783815</v>
+        <v>0.007724999999999999</v>
       </c>
       <c r="C26">
-        <v>0.008652449999999999</v>
+        <v>0.0083131</v>
       </c>
       <c r="D26">
-        <v>0.0058301</v>
+        <v>0.005540575</v>
       </c>
       <c r="E26">
-        <v>0.008776975000000001</v>
+        <v>0.0084936</v>
       </c>
       <c r="F26">
-        <v>0.00734695</v>
+        <v>0.007331525</v>
       </c>
       <c r="G26">
-        <v>0.007688925000000001</v>
+        <v>0.00748076</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1147,22 +1147,22 @@
         <v>32</v>
       </c>
       <c r="B27">
-        <v>0.007989</v>
+        <v>0.008093325</v>
       </c>
       <c r="C27">
-        <v>0.008886125</v>
+        <v>0.008559325000000001</v>
       </c>
       <c r="D27">
-        <v>0.005680899999999999</v>
+        <v>0.005566300000000001</v>
       </c>
       <c r="E27">
-        <v>0.008571499999999999</v>
+        <v>0.008343275000000001</v>
       </c>
       <c r="F27">
-        <v>0.007288149999999999</v>
+        <v>0.007203775</v>
       </c>
       <c r="G27">
-        <v>0.007683134999999999</v>
+        <v>0.0075532</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1170,22 +1170,22 @@
         <v>33</v>
       </c>
       <c r="B28">
-        <v>0.007420650000000001</v>
+        <v>0.007160175</v>
       </c>
       <c r="C28">
-        <v>0.0077784</v>
+        <v>0.007516324999999999</v>
       </c>
       <c r="D28">
-        <v>0.006293575</v>
+        <v>0.006166125</v>
       </c>
       <c r="E28">
-        <v>0.007590275</v>
+        <v>0.007366775</v>
       </c>
       <c r="F28">
-        <v>0.00594775</v>
+        <v>0.005700350000000001</v>
       </c>
       <c r="G28">
-        <v>0.007006130000000001</v>
+        <v>0.006781949999999999</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1193,22 +1193,22 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>0.010652425</v>
+        <v>0.010516325</v>
       </c>
       <c r="C29">
-        <v>0.04816585</v>
+        <v>0.04703395</v>
       </c>
       <c r="D29">
-        <v>0.026876925</v>
+        <v>0.02621945</v>
       </c>
       <c r="E29">
-        <v>0.009714350000000002</v>
+        <v>0.00954205</v>
       </c>
       <c r="F29">
-        <v>0.007708024999999999</v>
+        <v>0.007421975</v>
       </c>
       <c r="G29">
-        <v>0.020623515</v>
+        <v>0.02014675</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1216,22 +1216,22 @@
         <v>35</v>
       </c>
       <c r="B30">
-        <v>0.01632385</v>
+        <v>0.016441825</v>
       </c>
       <c r="C30">
-        <v>0.06030754999999999</v>
+        <v>0.05788620000000001</v>
       </c>
       <c r="D30">
-        <v>0.020156825</v>
+        <v>0.019103</v>
       </c>
       <c r="E30">
-        <v>0.009730925</v>
+        <v>0.009438599999999998</v>
       </c>
       <c r="F30">
-        <v>0.020242575</v>
+        <v>0.019814875</v>
       </c>
       <c r="G30">
-        <v>0.025352345</v>
+        <v>0.0245369</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1239,22 +1239,22 @@
         <v>36</v>
       </c>
       <c r="B31">
-        <v>0.01382505</v>
+        <v>0.013820225</v>
       </c>
       <c r="C31">
-        <v>0.05980769999999999</v>
+        <v>0.05753235</v>
       </c>
       <c r="D31">
-        <v>0.020428675</v>
+        <v>0.0196674</v>
       </c>
       <c r="E31">
-        <v>0.0091699</v>
+        <v>0.008816850000000001</v>
       </c>
       <c r="F31">
-        <v>0.01698675</v>
+        <v>0.01669665</v>
       </c>
       <c r="G31">
-        <v>0.024043615</v>
+        <v>0.023306695</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1262,22 +1262,22 @@
         <v>37</v>
       </c>
       <c r="B32">
-        <v>0.02566585</v>
+        <v>0.02554045</v>
       </c>
       <c r="C32">
-        <v>0.0320633</v>
+        <v>0.03139975</v>
       </c>
       <c r="D32">
-        <v>0.024742075</v>
+        <v>0.0236449</v>
       </c>
       <c r="E32">
-        <v>0.03337205</v>
+        <v>0.031760775</v>
       </c>
       <c r="F32">
-        <v>0.043375725</v>
+        <v>0.04162724999999999</v>
       </c>
       <c r="G32">
-        <v>0.0318438</v>
+        <v>0.030794625</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1285,22 +1285,22 @@
         <v>38</v>
       </c>
       <c r="B33">
-        <v>0.005563075</v>
+        <v>0.0056144</v>
       </c>
       <c r="C33">
-        <v>0.004078525</v>
+        <v>0.004153799999999999</v>
       </c>
       <c r="D33">
-        <v>0.003174600000000001</v>
+        <v>0.003070225</v>
       </c>
       <c r="E33">
-        <v>0.004179924999999999</v>
+        <v>0.004064725</v>
       </c>
       <c r="F33">
-        <v>0.008145100000000001</v>
+        <v>0.008104875000000001</v>
       </c>
       <c r="G33">
-        <v>0.005028245000000001</v>
+        <v>0.005001605</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1308,22 +1308,22 @@
         <v>39</v>
       </c>
       <c r="B34">
-        <v>0.008478099999999999</v>
+        <v>0.008455724999999999</v>
       </c>
       <c r="C34">
-        <v>0.00401885</v>
+        <v>0.003913625</v>
       </c>
       <c r="D34">
-        <v>0.0034743</v>
+        <v>0.003461575</v>
       </c>
       <c r="E34">
-        <v>0.003788425</v>
+        <v>0.003782225</v>
       </c>
       <c r="F34">
-        <v>0.008956200000000001</v>
+        <v>0.0089763</v>
       </c>
       <c r="G34">
-        <v>0.005743175000000001</v>
+        <v>0.00571789</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1331,22 +1331,22 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>0.005595149999999998</v>
+        <v>0.005878299999999999</v>
       </c>
       <c r="C35">
-        <v>0.0038784</v>
+        <v>0.00381805</v>
       </c>
       <c r="D35">
-        <v>0.00518475</v>
+        <v>0.00518875</v>
       </c>
       <c r="E35">
-        <v>0.003701149999999999</v>
+        <v>0.00360265</v>
       </c>
       <c r="F35">
-        <v>0.007603724999999999</v>
+        <v>0.007565350000000001</v>
       </c>
       <c r="G35">
-        <v>0.005192634999999999</v>
+        <v>0.00521062</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1354,22 +1354,22 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>0.002858175</v>
+        <v>0.002829949999999999</v>
       </c>
       <c r="C36">
-        <v>0.004120425</v>
+        <v>0.0040699</v>
       </c>
       <c r="D36">
-        <v>0.002676125</v>
+        <v>0.002607025</v>
       </c>
       <c r="E36">
-        <v>0.003049325</v>
+        <v>0.002956325</v>
       </c>
       <c r="F36">
-        <v>0.005155775</v>
+        <v>0.005150975</v>
       </c>
       <c r="G36">
-        <v>0.003571965</v>
+        <v>0.003522834999999999</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1377,22 +1377,22 @@
         <v>42</v>
       </c>
       <c r="B37">
-        <v>0.003613575</v>
+        <v>0.00358465</v>
       </c>
       <c r="C37">
-        <v>0.004256175000000001</v>
+        <v>0.0042121</v>
       </c>
       <c r="D37">
-        <v>0.0034929</v>
+        <v>0.0033971</v>
       </c>
       <c r="E37">
-        <v>0.002814225</v>
+        <v>0.002787175</v>
       </c>
       <c r="F37">
-        <v>0.004682575</v>
+        <v>0.00463045</v>
       </c>
       <c r="G37">
-        <v>0.00377189</v>
+        <v>0.003722295</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1400,22 +1400,22 @@
         <v>43</v>
       </c>
       <c r="B38">
-        <v>0.004869825</v>
+        <v>0.004833325</v>
       </c>
       <c r="C38">
-        <v>0.004739125</v>
+        <v>0.00463145</v>
       </c>
       <c r="D38">
-        <v>0.004987275</v>
+        <v>0.004861625</v>
       </c>
       <c r="E38">
-        <v>0.004925525</v>
+        <v>0.004861375</v>
       </c>
       <c r="F38">
-        <v>0.008264825</v>
+        <v>0.00811835</v>
       </c>
       <c r="G38">
-        <v>0.005557315</v>
+        <v>0.005461225</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1423,22 +1423,22 @@
         <v>44</v>
       </c>
       <c r="B39">
-        <v>0.00566075</v>
+        <v>0.00553905</v>
       </c>
       <c r="C39">
-        <v>0.017067475</v>
+        <v>0.016621725</v>
       </c>
       <c r="D39">
-        <v>0.009290349999999999</v>
+        <v>0.008725499999999999</v>
       </c>
       <c r="E39">
-        <v>0.0047869</v>
+        <v>0.004607675</v>
       </c>
       <c r="F39">
-        <v>0.0032086</v>
+        <v>0.003043875</v>
       </c>
       <c r="G39">
-        <v>0.008002814999999998</v>
+        <v>0.007707565</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1446,22 +1446,22 @@
         <v>45</v>
       </c>
       <c r="B40">
-        <v>0.010092175</v>
+        <v>0.010108025</v>
       </c>
       <c r="C40">
-        <v>0.0272685</v>
+        <v>0.02624135</v>
       </c>
       <c r="D40">
-        <v>0.011962775</v>
+        <v>0.01107915</v>
       </c>
       <c r="E40">
-        <v>0.005414675</v>
+        <v>0.0053021</v>
       </c>
       <c r="F40">
-        <v>0.011559675</v>
+        <v>0.0112927</v>
       </c>
       <c r="G40">
-        <v>0.01325956</v>
+        <v>0.012804665</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1469,22 +1469,22 @@
         <v>46</v>
       </c>
       <c r="B41">
-        <v>0.008499949999999999</v>
+        <v>0.008642149999999999</v>
       </c>
       <c r="C41">
-        <v>0.027297</v>
+        <v>0.0261051</v>
       </c>
       <c r="D41">
-        <v>0.01124555</v>
+        <v>0.0106154</v>
       </c>
       <c r="E41">
-        <v>0.005200475</v>
+        <v>0.005131500000000001</v>
       </c>
       <c r="F41">
-        <v>0.009091575000000001</v>
+        <v>0.009022299999999999</v>
       </c>
       <c r="G41">
-        <v>0.01226691</v>
+        <v>0.01190329</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1492,22 +1492,22 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>0.008465425</v>
+        <v>0.008134124999999999</v>
       </c>
       <c r="C42">
-        <v>0.009256250000000001</v>
+        <v>0.00882465</v>
       </c>
       <c r="D42">
-        <v>0.00608025</v>
+        <v>0.005791474999999999</v>
       </c>
       <c r="E42">
-        <v>0.008823900000000001</v>
+        <v>0.008921100000000001</v>
       </c>
       <c r="F42">
-        <v>0.007745674999999999</v>
+        <v>0.007520674999999999</v>
       </c>
       <c r="G42">
-        <v>0.0080743</v>
+        <v>0.007838405</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1515,22 +1515,22 @@
         <v>48</v>
       </c>
       <c r="B43">
-        <v>0.0141081</v>
+        <v>0.0141256</v>
       </c>
       <c r="C43">
-        <v>0.0599003</v>
+        <v>0.05748179999999999</v>
       </c>
       <c r="D43">
-        <v>0.02065529999999999</v>
+        <v>0.01950055</v>
       </c>
       <c r="E43">
-        <v>0.009409899999999999</v>
+        <v>0.009166849999999999</v>
       </c>
       <c r="F43">
-        <v>0.017254525</v>
+        <v>0.016954</v>
       </c>
       <c r="G43">
-        <v>0.024265625</v>
+        <v>0.02344576</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1538,22 +1538,22 @@
         <v>49</v>
       </c>
       <c r="B44">
-        <v>0.005646674999999999</v>
+        <v>0.0055933</v>
       </c>
       <c r="C44">
-        <v>0.00419345</v>
+        <v>0.004103525</v>
       </c>
       <c r="D44">
-        <v>0.003250975</v>
+        <v>0.003165425</v>
       </c>
       <c r="E44">
-        <v>0.00427745</v>
+        <v>0.004178825000000001</v>
       </c>
       <c r="F44">
-        <v>0.008234150000000001</v>
+        <v>0.00810755</v>
       </c>
       <c r="G44">
-        <v>0.00512054</v>
+        <v>0.005029725000000001</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1561,22 +1561,22 @@
         <v>50</v>
       </c>
       <c r="B45">
-        <v>0.0060334</v>
+        <v>0.006123324999999999</v>
       </c>
       <c r="C45">
-        <v>0.004473575</v>
+        <v>0.00459715</v>
       </c>
       <c r="D45">
-        <v>0.0038815</v>
+        <v>0.0037878</v>
       </c>
       <c r="E45">
-        <v>0.00411905</v>
+        <v>0.003869549999999999</v>
       </c>
       <c r="F45">
-        <v>0.008536599999999998</v>
+        <v>0.0084998</v>
       </c>
       <c r="G45">
-        <v>0.005408825</v>
+        <v>0.005375525000000001</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1584,22 +1584,22 @@
         <v>51</v>
       </c>
       <c r="B46">
-        <v>0.008640600000000002</v>
+        <v>0.00855885</v>
       </c>
       <c r="C46">
-        <v>0.004088325</v>
+        <v>0.004022825</v>
       </c>
       <c r="D46">
-        <v>0.0036034</v>
+        <v>0.003522525</v>
       </c>
       <c r="E46">
-        <v>0.0038975</v>
+        <v>0.003783225</v>
       </c>
       <c r="F46">
-        <v>0.009158099999999999</v>
+        <v>0.008915724999999999</v>
       </c>
       <c r="G46">
-        <v>0.005877584999999999</v>
+        <v>0.00576063</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -1607,22 +1607,22 @@
         <v>52</v>
       </c>
       <c r="B47">
-        <v>0.00363435</v>
+        <v>0.003643975</v>
       </c>
       <c r="C47">
-        <v>0.0043871</v>
+        <v>0.0042112</v>
       </c>
       <c r="D47">
-        <v>0.0035842</v>
+        <v>0.00348915</v>
       </c>
       <c r="E47">
-        <v>0.0029311</v>
+        <v>0.002819625</v>
       </c>
       <c r="F47">
-        <v>0.00468885</v>
+        <v>0.00465595</v>
       </c>
       <c r="G47">
-        <v>0.003845119999999999</v>
+        <v>0.003763979999999999</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -1630,22 +1630,22 @@
         <v>53</v>
       </c>
       <c r="B48">
-        <v>0.0087245</v>
+        <v>0.008533275</v>
       </c>
       <c r="C48">
-        <v>0.027567875</v>
+        <v>0.02636425</v>
       </c>
       <c r="D48">
-        <v>0.0116931</v>
+        <v>0.011042775</v>
       </c>
       <c r="E48">
-        <v>0.005508375</v>
+        <v>0.00536295</v>
       </c>
       <c r="F48">
-        <v>0.009623100000000001</v>
+        <v>0.009244024999999999</v>
       </c>
       <c r="G48">
-        <v>0.01262339</v>
+        <v>0.012109455</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -1653,22 +1653,22 @@
         <v>54</v>
       </c>
       <c r="B49">
-        <v>0.00616065</v>
+        <v>0.006097749999999999</v>
       </c>
       <c r="C49">
-        <v>0.004594325</v>
+        <v>0.0046258</v>
       </c>
       <c r="D49">
-        <v>0.004005175</v>
+        <v>0.003862475</v>
       </c>
       <c r="E49">
-        <v>0.0039245</v>
+        <v>0.003937475</v>
       </c>
       <c r="F49">
-        <v>0.008776600000000001</v>
+        <v>0.008391375</v>
       </c>
       <c r="G49">
-        <v>0.00549225</v>
+        <v>0.005382975</v>
       </c>
     </row>
   </sheetData>
@@ -1824,22 +1824,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>9.25</v>
+        <v>6.5</v>
       </c>
       <c r="C7">
-        <v>10.25</v>
+        <v>8</v>
       </c>
       <c r="D7">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E7">
-        <v>9.5</v>
+        <v>8</v>
       </c>
       <c r="F7">
         <v>4</v>
       </c>
       <c r="G7">
-        <v>9.199999999999999</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1916,22 +1916,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>8.75</v>
+        <v>6.25</v>
       </c>
       <c r="C11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11">
-        <v>15.25</v>
+        <v>13</v>
       </c>
       <c r="E11">
-        <v>10.25</v>
+        <v>8.25</v>
       </c>
       <c r="F11">
         <v>4</v>
       </c>
       <c r="G11">
-        <v>9.65</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1962,22 +1962,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>9.5</v>
+        <v>7.75</v>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>8.75</v>
       </c>
       <c r="D13">
-        <v>16.75</v>
+        <v>14.25</v>
       </c>
       <c r="E13">
-        <v>9.75</v>
+        <v>8</v>
       </c>
       <c r="F13">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="G13">
-        <v>10.7</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2031,22 +2031,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>10.25</v>
+        <v>8.25</v>
       </c>
       <c r="C16">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D16">
-        <v>15</v>
+        <v>12.75</v>
       </c>
       <c r="E16">
-        <v>11.25</v>
+        <v>8.5</v>
       </c>
       <c r="F16">
         <v>4</v>
       </c>
       <c r="G16">
-        <v>10.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -2146,22 +2146,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C21">
-        <v>11</v>
+        <v>8.5</v>
       </c>
       <c r="D21">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="E21">
-        <v>10</v>
+        <v>8.5</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="G21">
-        <v>9.6</v>
+        <v>8.050000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2169,22 +2169,22 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>9.25</v>
+        <v>6.75</v>
       </c>
       <c r="C22">
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="D22">
-        <v>13.5</v>
+        <v>11.25</v>
       </c>
       <c r="E22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22">
         <v>4</v>
       </c>
       <c r="G22">
-        <v>9.25</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -2192,22 +2192,22 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>10</v>
+        <v>7.25</v>
       </c>
       <c r="C23">
-        <v>11.25</v>
+        <v>8.5</v>
       </c>
       <c r="D23">
-        <v>16.5</v>
+        <v>14.25</v>
       </c>
       <c r="E23">
-        <v>9.25</v>
+        <v>8</v>
       </c>
       <c r="F23">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="G23">
-        <v>10.7</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -2261,22 +2261,22 @@
         <v>31</v>
       </c>
       <c r="B26">
+        <v>8.5</v>
+      </c>
+      <c r="C26">
         <v>10.75</v>
       </c>
-      <c r="C26">
-        <v>12.25</v>
-      </c>
       <c r="D26">
-        <v>16.75</v>
+        <v>15.5</v>
       </c>
       <c r="E26">
-        <v>10</v>
+        <v>8.5</v>
       </c>
       <c r="F26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G26">
-        <v>11.35</v>
+        <v>9.85</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2307,22 +2307,22 @@
         <v>33</v>
       </c>
       <c r="B28">
-        <v>8.75</v>
+        <v>6.25</v>
       </c>
       <c r="C28">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D28">
-        <v>15</v>
+        <v>12.75</v>
       </c>
       <c r="E28">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F28">
         <v>4</v>
       </c>
       <c r="G28">
-        <v>9.75</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2330,22 +2330,22 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>8.75</v>
+        <v>7.5</v>
       </c>
       <c r="C29">
-        <v>11</v>
+        <v>8.5</v>
       </c>
       <c r="D29">
-        <v>15.75</v>
+        <v>14.25</v>
       </c>
       <c r="E29">
-        <v>9.5</v>
+        <v>8.25</v>
       </c>
       <c r="F29">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="G29">
-        <v>10.25</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2353,22 +2353,22 @@
         <v>35</v>
       </c>
       <c r="B30">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="C30">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="D30">
-        <v>16.5</v>
+        <v>14.75</v>
       </c>
       <c r="E30">
-        <v>9.25</v>
+        <v>7.75</v>
       </c>
       <c r="F30">
-        <v>7.25</v>
+        <v>6.25</v>
       </c>
       <c r="G30">
-        <v>10.7</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2399,22 +2399,22 @@
         <v>37</v>
       </c>
       <c r="B32">
-        <v>10.25</v>
+        <v>8.25</v>
       </c>
       <c r="C32">
-        <v>10.75</v>
+        <v>9.25</v>
       </c>
       <c r="D32">
-        <v>15</v>
+        <v>12.75</v>
       </c>
       <c r="E32">
-        <v>11.25</v>
+        <v>8.5</v>
       </c>
       <c r="F32">
         <v>4</v>
       </c>
       <c r="G32">
-        <v>10.25</v>
+        <v>8.550000000000001</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2468,22 +2468,22 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C35">
-        <v>11</v>
+        <v>7.75</v>
       </c>
       <c r="D35">
-        <v>15</v>
+        <v>12.75</v>
       </c>
       <c r="E35">
-        <v>9</v>
+        <v>7.75</v>
       </c>
       <c r="F35">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="G35">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -2491,22 +2491,22 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>8</v>
+        <v>6.25</v>
       </c>
       <c r="C36">
-        <v>12.5</v>
+        <v>10.5</v>
       </c>
       <c r="D36">
-        <v>15.5</v>
+        <v>14.25</v>
       </c>
       <c r="E36">
-        <v>10.25</v>
+        <v>6.75</v>
       </c>
       <c r="F36">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G36">
-        <v>10.6</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2537,22 +2537,22 @@
         <v>43</v>
       </c>
       <c r="B38">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C38">
-        <v>10.5</v>
+        <v>8.25</v>
       </c>
       <c r="D38">
-        <v>15</v>
+        <v>14.25</v>
       </c>
       <c r="E38">
-        <v>11.25</v>
+        <v>8.75</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="G38">
-        <v>9.75</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -2560,22 +2560,22 @@
         <v>44</v>
       </c>
       <c r="B39">
-        <v>9.25</v>
+        <v>7.25</v>
       </c>
       <c r="C39">
-        <v>11</v>
+        <v>8.5</v>
       </c>
       <c r="D39">
-        <v>15.75</v>
+        <v>14.25</v>
       </c>
       <c r="E39">
-        <v>9.25</v>
+        <v>8.25</v>
       </c>
       <c r="F39">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="G39">
-        <v>10.3</v>
+        <v>8.85</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2583,22 +2583,22 @@
         <v>45</v>
       </c>
       <c r="B40">
-        <v>10.75</v>
+        <v>7.25</v>
       </c>
       <c r="C40">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="D40">
-        <v>16.5</v>
+        <v>14.75</v>
       </c>
       <c r="E40">
-        <v>9</v>
+        <v>7.75</v>
       </c>
       <c r="F40">
-        <v>7.25</v>
+        <v>6.25</v>
       </c>
       <c r="G40">
-        <v>10.9</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -2629,22 +2629,22 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C42">
-        <v>11.75</v>
+        <v>10.5</v>
       </c>
       <c r="D42">
-        <v>16.75</v>
+        <v>15.5</v>
       </c>
       <c r="E42">
-        <v>10</v>
+        <v>8.5</v>
       </c>
       <c r="F42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G42">
-        <v>11.3</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -2652,22 +2652,22 @@
         <v>48</v>
       </c>
       <c r="B43">
+        <v>7.5</v>
+      </c>
+      <c r="C43">
         <v>9</v>
       </c>
-      <c r="C43">
-        <v>10.5</v>
-      </c>
       <c r="D43">
-        <v>16.75</v>
+        <v>14.75</v>
       </c>
       <c r="E43">
-        <v>9</v>
+        <v>7.75</v>
       </c>
       <c r="F43">
-        <v>7</v>
+        <v>6.25</v>
       </c>
       <c r="G43">
-        <v>10.45</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -2675,22 +2675,22 @@
         <v>49</v>
       </c>
       <c r="B44">
+        <v>6.75</v>
+      </c>
+      <c r="C44">
         <v>8.75</v>
       </c>
-      <c r="C44">
-        <v>12</v>
-      </c>
       <c r="D44">
-        <v>15</v>
+        <v>12.75</v>
       </c>
       <c r="E44">
-        <v>11.25</v>
+        <v>8.5</v>
       </c>
       <c r="F44">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="G44">
-        <v>10.65</v>
+        <v>8.550000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -2721,22 +2721,22 @@
         <v>51</v>
       </c>
       <c r="B46">
+        <v>7</v>
+      </c>
+      <c r="C46">
         <v>9</v>
       </c>
-      <c r="C46">
-        <v>12.25</v>
-      </c>
       <c r="D46">
-        <v>16</v>
+        <v>14.5</v>
       </c>
       <c r="E46">
-        <v>9.25</v>
+        <v>7.75</v>
       </c>
       <c r="F46">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G46">
-        <v>10.65</v>
+        <v>8.85</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -2744,22 +2744,22 @@
         <v>52</v>
       </c>
       <c r="B47">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C47">
-        <v>12</v>
+        <v>9.5</v>
       </c>
       <c r="D47">
-        <v>16.5</v>
+        <v>15.25</v>
       </c>
       <c r="E47">
-        <v>9.75</v>
+        <v>8.5</v>
       </c>
       <c r="F47">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G47">
-        <v>10.6</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2767,22 +2767,22 @@
         <v>53</v>
       </c>
       <c r="B48">
+        <v>7.25</v>
+      </c>
+      <c r="C48">
         <v>9.5</v>
       </c>
-      <c r="C48">
-        <v>11</v>
-      </c>
       <c r="D48">
-        <v>16.75</v>
+        <v>14.75</v>
       </c>
       <c r="E48">
-        <v>9</v>
+        <v>7.75</v>
       </c>
       <c r="F48">
-        <v>7</v>
+        <v>6.25</v>
       </c>
       <c r="G48">
-        <v>10.65</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -2790,22 +2790,22 @@
         <v>54</v>
       </c>
       <c r="B49">
+        <v>7</v>
+      </c>
+      <c r="C49">
         <v>9</v>
       </c>
-      <c r="C49">
-        <v>12.25</v>
-      </c>
       <c r="D49">
-        <v>16</v>
+        <v>14.5</v>
       </c>
       <c r="E49">
-        <v>9.75</v>
+        <v>8.25</v>
       </c>
       <c r="F49">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G49">
-        <v>10.75</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2961,22 +2961,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>91.72485257725916</v>
+        <v>89.13939731950015</v>
       </c>
       <c r="C7">
-        <v>94.28719018831526</v>
+        <v>92.92004125279729</v>
       </c>
       <c r="D7">
-        <v>96.09135241389544</v>
+        <v>94.65664671106151</v>
       </c>
       <c r="E7">
-        <v>89.60451849562072</v>
+        <v>88.12126645620715</v>
       </c>
       <c r="F7">
         <v>87.33691238960859</v>
       </c>
       <c r="G7">
-        <v>91.80896521293984</v>
+        <v>90.43485282583494</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3053,22 +3053,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>90.54621526063178</v>
+        <v>88.81605475511716</v>
       </c>
       <c r="C11">
-        <v>92.52641660713583</v>
+        <v>92.35155128758481</v>
       </c>
       <c r="D11">
-        <v>95.79404337902628</v>
+        <v>94.77232629366651</v>
       </c>
       <c r="E11">
-        <v>88.20410850128535</v>
+        <v>87.44194575170043</v>
       </c>
       <c r="F11">
         <v>87.83084116930945</v>
       </c>
       <c r="G11">
-        <v>90.98032498347774</v>
+        <v>90.24254385147567</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -3099,22 +3099,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>89.5194338638298</v>
+        <v>89.22701017523383</v>
       </c>
       <c r="C13">
-        <v>95.55804687106941</v>
+        <v>94.92412607931394</v>
       </c>
       <c r="D13">
-        <v>101.8589186747198</v>
+        <v>99.63732995997091</v>
       </c>
       <c r="E13">
-        <v>89.35311325426825</v>
+        <v>88.58420760391871</v>
       </c>
       <c r="F13">
-        <v>90.29777793799398</v>
+        <v>90.05714420705036</v>
       </c>
       <c r="G13">
-        <v>93.31745812037624</v>
+        <v>92.48596360509755</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -3168,22 +3168,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>88.99921179650484</v>
+        <v>88.57888496415744</v>
       </c>
       <c r="C16">
-        <v>93.01525638432572</v>
+        <v>92.3043155870872</v>
       </c>
       <c r="D16">
-        <v>95.24546858635269</v>
+        <v>94.42117856929082</v>
       </c>
       <c r="E16">
-        <v>87.02915991771309</v>
+        <v>86.50435909119437</v>
       </c>
       <c r="F16">
         <v>87.25337971078574</v>
       </c>
       <c r="G16">
-        <v>90.30849527913641</v>
+        <v>89.81242358450312</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -3283,22 +3283,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>94.42209588551708</v>
+        <v>91.1611041251298</v>
       </c>
       <c r="C21">
-        <v>96.0303354056141</v>
+        <v>93.72825760107301</v>
       </c>
       <c r="D21">
-        <v>98.25915590201265</v>
+        <v>98.15890054347378</v>
       </c>
       <c r="E21">
-        <v>89.70359386802247</v>
+        <v>88.73381198849388</v>
       </c>
       <c r="F21">
-        <v>89.17676618598557</v>
+        <v>88.98646867694093</v>
       </c>
       <c r="G21">
-        <v>93.51838944943037</v>
+        <v>92.15370858702228</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -3306,22 +3306,22 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>90.93685523906024</v>
+        <v>89.2776595859244</v>
       </c>
       <c r="C22">
-        <v>93.91391810676384</v>
+        <v>92.90307720918985</v>
       </c>
       <c r="D22">
-        <v>95.40427079958275</v>
+        <v>94.41051680500189</v>
       </c>
       <c r="E22">
-        <v>89.52248109096848</v>
+        <v>88.1854601545144</v>
       </c>
       <c r="F22">
         <v>87.38393931334436</v>
       </c>
       <c r="G22">
-        <v>91.43229290994392</v>
+        <v>90.43213061359498</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -3329,22 +3329,22 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>89.6159900426394</v>
+        <v>89.22701017523383</v>
       </c>
       <c r="C23">
-        <v>94.74917278692931</v>
+        <v>94.66869395521077</v>
       </c>
       <c r="D23">
-        <v>100.9296464662099</v>
+        <v>98.53898956548846</v>
       </c>
       <c r="E23">
-        <v>89.60108077810561</v>
+        <v>88.86499004755807</v>
       </c>
       <c r="F23">
-        <v>87.91636272147292</v>
+        <v>87.85248644886262</v>
       </c>
       <c r="G23">
-        <v>92.56245055907142</v>
+        <v>91.83043403847076</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -3398,22 +3398,22 @@
         <v>31</v>
       </c>
       <c r="B26">
-        <v>89.14083905815238</v>
+        <v>88.75888657103675</v>
       </c>
       <c r="C26">
-        <v>97.03251914740976</v>
+        <v>97.00780758575567</v>
       </c>
       <c r="D26">
-        <v>97.77239606356295</v>
+        <v>97.64968979182635</v>
       </c>
       <c r="E26">
-        <v>89.04474251239938</v>
+        <v>88.86499004755807</v>
       </c>
       <c r="F26">
-        <v>89.2164034626815</v>
+        <v>88.62102407633546</v>
       </c>
       <c r="G26">
-        <v>92.4413800488412</v>
+        <v>92.18047961450246</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -3444,22 +3444,22 @@
         <v>33</v>
       </c>
       <c r="B28">
-        <v>90.54114361467967</v>
+        <v>89.12431128621597</v>
       </c>
       <c r="C28">
-        <v>92.8466097608916</v>
+        <v>92.35632712783598</v>
       </c>
       <c r="D28">
-        <v>95.82890158590824</v>
+        <v>94.39401605200109</v>
       </c>
       <c r="E28">
-        <v>89.72300720183679</v>
+        <v>88.88690818712263</v>
       </c>
       <c r="F28">
         <v>87.25337971078574</v>
       </c>
       <c r="G28">
-        <v>91.2386083748204</v>
+        <v>90.40298847279227</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -3467,22 +3467,22 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>89.54733577687858</v>
+        <v>88.89834825349419</v>
       </c>
       <c r="C29">
-        <v>96.12967005510683</v>
+        <v>94.58157556205583</v>
       </c>
       <c r="D29">
-        <v>103.4295116012851</v>
+        <v>102.1853912455699</v>
       </c>
       <c r="E29">
-        <v>89.35350062346056</v>
+        <v>88.58420760391871</v>
       </c>
       <c r="F29">
-        <v>90.58368323137562</v>
+        <v>90.14531001978574</v>
       </c>
       <c r="G29">
-        <v>93.80874025762134</v>
+        <v>92.87896653696487</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -3490,22 +3490,22 @@
         <v>35</v>
       </c>
       <c r="B30">
-        <v>90.03093966588489</v>
+        <v>88.98799547445716</v>
       </c>
       <c r="C30">
-        <v>97.12757998731722</v>
+        <v>96.23340722565031</v>
       </c>
       <c r="D30">
-        <v>98.95532963718236</v>
+        <v>98.3909295861728</v>
       </c>
       <c r="E30">
-        <v>89.38253734231658</v>
+        <v>88.59805700955056</v>
       </c>
       <c r="F30">
-        <v>92.69865149093101</v>
+        <v>92.13466900158528</v>
       </c>
       <c r="G30">
-        <v>93.63900762472642</v>
+        <v>92.86901165948322</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -3536,22 +3536,22 @@
         <v>37</v>
       </c>
       <c r="B32">
-        <v>88.99921179650484</v>
+        <v>88.57888496415744</v>
       </c>
       <c r="C32">
-        <v>93.84773767906115</v>
+        <v>93.24939669889704</v>
       </c>
       <c r="D32">
-        <v>95.24546858635269</v>
+        <v>94.42117856929082</v>
       </c>
       <c r="E32">
-        <v>87.02915991771309</v>
+        <v>86.50435909119437</v>
       </c>
       <c r="F32">
         <v>87.25337971078574</v>
       </c>
       <c r="G32">
-        <v>90.4749915380835</v>
+        <v>90.00143980686508</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -3605,22 +3605,22 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>92.86734279435822</v>
+        <v>91.10993454476508</v>
       </c>
       <c r="C35">
-        <v>94.72051092461355</v>
+        <v>92.29928073650612</v>
       </c>
       <c r="D35">
-        <v>96.2945479532705</v>
+        <v>96.01541363581259</v>
       </c>
       <c r="E35">
-        <v>89.63197465251324</v>
+        <v>88.86857894582849</v>
       </c>
       <c r="F35">
-        <v>87.25337971078574</v>
+        <v>87.0681506715672</v>
       </c>
       <c r="G35">
-        <v>92.15355120710825</v>
+        <v>91.07227170689589</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -3628,22 +3628,22 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>97.42466324028555</v>
+        <v>95.43566511011795</v>
       </c>
       <c r="C36">
-        <v>101.0884357896212</v>
+        <v>99.02144924571451</v>
       </c>
       <c r="D36">
-        <v>98.75915590201265</v>
+        <v>98.52857770962854</v>
       </c>
       <c r="E36">
-        <v>91.5118722934187</v>
+        <v>88.88470486692829</v>
       </c>
       <c r="F36">
-        <v>91.29592613104968</v>
+        <v>89.4557226091525</v>
       </c>
       <c r="G36">
-        <v>96.01601067127756</v>
+        <v>94.26522390830834</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -3674,22 +3674,22 @@
         <v>43</v>
       </c>
       <c r="B38">
-        <v>93.08600399896729</v>
+        <v>90.74289877000135</v>
       </c>
       <c r="C38">
-        <v>96.17678201502082</v>
+        <v>93.91924060669805</v>
       </c>
       <c r="D38">
-        <v>98.25915590201265</v>
+        <v>98.12554671335766</v>
       </c>
       <c r="E38">
-        <v>88.47938871750956</v>
+        <v>87.00466654293592</v>
       </c>
       <c r="F38">
-        <v>89.17676618598557</v>
+        <v>88.98646867694093</v>
       </c>
       <c r="G38">
-        <v>93.03561936389917</v>
+        <v>91.75576426198678</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -3697,22 +3697,22 @@
         <v>44</v>
       </c>
       <c r="B39">
-        <v>89.60406067016351</v>
+        <v>88.89834825349419</v>
       </c>
       <c r="C39">
-        <v>95.76906682557187</v>
+        <v>94.59092271771277</v>
       </c>
       <c r="D39">
-        <v>102.1639796876998</v>
+        <v>100.8161412879935</v>
       </c>
       <c r="E39">
-        <v>89.63438094807063</v>
+        <v>88.91691119506876</v>
       </c>
       <c r="F39">
-        <v>87.91636272147292</v>
+        <v>87.85248644886262</v>
       </c>
       <c r="G39">
-        <v>93.01757017059575</v>
+        <v>92.21496198062638</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -3720,22 +3720,22 @@
         <v>45</v>
       </c>
       <c r="B40">
-        <v>90.65444921294146</v>
+        <v>89.0003034744495</v>
       </c>
       <c r="C40">
-        <v>97.51119481579398</v>
+        <v>96.75656827501791</v>
       </c>
       <c r="D40">
-        <v>98.76494818645951</v>
+        <v>98.20054813544995</v>
       </c>
       <c r="E40">
-        <v>89.60108077810561</v>
+        <v>88.86499004755807</v>
       </c>
       <c r="F40">
-        <v>92.55515667937578</v>
+        <v>92.13301812599349</v>
       </c>
       <c r="G40">
-        <v>93.81736593453527</v>
+        <v>92.99108561169378</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -3766,22 +3766,22 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>89.17692153974153</v>
+        <v>88.97492867645308</v>
       </c>
       <c r="C42">
-        <v>97.06542392572945</v>
+        <v>97.05189493017757</v>
       </c>
       <c r="D42">
-        <v>97.89291056653599</v>
+        <v>97.77020429479941</v>
       </c>
       <c r="E42">
-        <v>89.04474251239938</v>
+        <v>88.86499004755807</v>
       </c>
       <c r="F42">
-        <v>89.2164034626815</v>
+        <v>88.62102407633546</v>
       </c>
       <c r="G42">
-        <v>92.47928040141757</v>
+        <v>92.25660840506472</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -3789,22 +3789,22 @@
         <v>48</v>
       </c>
       <c r="B43">
-        <v>89.45770732525547</v>
+        <v>88.89834825349419</v>
       </c>
       <c r="C43">
-        <v>97.12757998731722</v>
+        <v>96.23340722565031</v>
       </c>
       <c r="D43">
-        <v>99.50277513396722</v>
+        <v>98.65358861299265</v>
       </c>
       <c r="E43">
-        <v>89.34618134646816</v>
+        <v>88.58420760391871</v>
       </c>
       <c r="F43">
-        <v>91.43396250283749</v>
+        <v>90.57933017944244</v>
       </c>
       <c r="G43">
-        <v>93.3736412591691</v>
+        <v>92.58977637509966</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -3812,22 +3812,22 @@
         <v>49</v>
       </c>
       <c r="B44">
-        <v>97.61169407182825</v>
+        <v>95.63997164837502</v>
       </c>
       <c r="C44">
-        <v>98.37401427221501</v>
+        <v>96.60137900637835</v>
       </c>
       <c r="D44">
-        <v>97.14647937060019</v>
+        <v>96.86734505314232</v>
       </c>
       <c r="E44">
-        <v>88.00534867131728</v>
+        <v>87.06506325136354</v>
       </c>
       <c r="F44">
-        <v>90.50304247160911</v>
+        <v>90.40120411245863</v>
       </c>
       <c r="G44">
-        <v>94.32811577151396</v>
+        <v>93.31499261434357</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -3858,22 +3858,22 @@
         <v>51</v>
       </c>
       <c r="B46">
-        <v>92.86734279435822</v>
+        <v>91.10993454476508</v>
       </c>
       <c r="C46">
-        <v>98.62237109481013</v>
+        <v>96.87551720889043</v>
       </c>
       <c r="D46">
-        <v>100.3085436257117</v>
+        <v>100.1769997821878</v>
       </c>
       <c r="E46">
-        <v>89.44302272585969</v>
+        <v>88.65353820228947</v>
       </c>
       <c r="F46">
-        <v>89.63303155760246</v>
+        <v>89.61956084446015</v>
       </c>
       <c r="G46">
-        <v>94.17486235966844</v>
+        <v>93.28711011651858</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -3881,22 +3881,22 @@
         <v>52</v>
       </c>
       <c r="B47">
-        <v>93.08600399896729</v>
+        <v>90.74289877000135</v>
       </c>
       <c r="C47">
-        <v>99.84825346925018</v>
+        <v>97.71788715626477</v>
       </c>
       <c r="D47">
-        <v>100.9307287772664</v>
+        <v>100.7001505848823</v>
       </c>
       <c r="E47">
-        <v>92.21947187576669</v>
+        <v>91.51690837354806</v>
       </c>
       <c r="F47">
-        <v>91.29592613104968</v>
+        <v>89.4557226091525</v>
       </c>
       <c r="G47">
-        <v>95.47607685046005</v>
+        <v>94.02671349876979</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -3904,22 +3904,22 @@
         <v>53</v>
       </c>
       <c r="B48">
-        <v>89.73341899102348</v>
+        <v>88.89834825349419</v>
       </c>
       <c r="C48">
-        <v>97.51119481579398</v>
+        <v>96.75656827501791</v>
       </c>
       <c r="D48">
-        <v>99.31239368324435</v>
+        <v>98.46320716226978</v>
       </c>
       <c r="E48">
-        <v>89.60108077810561</v>
+        <v>88.86499004755807</v>
       </c>
       <c r="F48">
-        <v>91.1329880230457</v>
+        <v>90.3710000566772</v>
       </c>
       <c r="G48">
-        <v>93.45821525824263</v>
+        <v>92.67082275900343</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -3927,22 +3927,22 @@
         <v>54</v>
       </c>
       <c r="B49">
-        <v>92.86734279435822</v>
+        <v>91.10993454476508</v>
       </c>
       <c r="C49">
-        <v>98.62237109481013</v>
+        <v>96.87551720889043</v>
       </c>
       <c r="D49">
-        <v>100.3085436257117</v>
+        <v>100.1658172160856</v>
       </c>
       <c r="E49">
-        <v>91.26310109453651</v>
+        <v>90.49970538785178</v>
       </c>
       <c r="F49">
-        <v>89.86604866666633</v>
+        <v>89.8428632552461</v>
       </c>
       <c r="G49">
-        <v>94.58548145521658</v>
+        <v>93.69876752256781</v>
       </c>
     </row>
   </sheetData>
@@ -6372,22 +6372,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>7.25</v>
+        <v>4.5</v>
       </c>
       <c r="C7">
-        <v>8.25</v>
+        <v>6</v>
       </c>
       <c r="D7">
-        <v>11</v>
+        <v>8.75</v>
       </c>
       <c r="E7">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7">
-        <v>7.2</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -6464,22 +6464,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>6.75</v>
+        <v>4.25</v>
       </c>
       <c r="C11">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E11">
-        <v>7.75</v>
+        <v>6</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
       <c r="G11">
-        <v>7.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -6510,22 +6510,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>7.5</v>
+        <v>5.25</v>
       </c>
       <c r="C13">
-        <v>9</v>
+        <v>6.75</v>
       </c>
       <c r="D13">
-        <v>14.75</v>
+        <v>12.25</v>
       </c>
       <c r="E13">
-        <v>7.5</v>
+        <v>5.75</v>
       </c>
       <c r="F13">
         <v>4</v>
       </c>
       <c r="G13">
-        <v>8.550000000000001</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -6579,22 +6579,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>8.25</v>
+        <v>5.5</v>
       </c>
       <c r="C16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E16">
-        <v>9.25</v>
+        <v>6.5</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>8.1</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -6694,22 +6694,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C21">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="D21">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="E21">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="G21">
-        <v>7.6</v>
+        <v>6.05</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -6717,22 +6717,22 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>7.25</v>
+        <v>4.75</v>
       </c>
       <c r="C22">
-        <v>8.25</v>
+        <v>6</v>
       </c>
       <c r="D22">
-        <v>11.5</v>
+        <v>9.25</v>
       </c>
       <c r="E22">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F22">
         <v>2</v>
       </c>
       <c r="G22">
-        <v>7.2</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -6740,22 +6740,22 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>8</v>
+        <v>5.25</v>
       </c>
       <c r="C23">
-        <v>9.25</v>
+        <v>6.5</v>
       </c>
       <c r="D23">
-        <v>14.5</v>
+        <v>12.25</v>
       </c>
       <c r="E23">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F23">
         <v>4</v>
       </c>
       <c r="G23">
-        <v>8.550000000000001</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -6809,22 +6809,22 @@
         <v>31</v>
       </c>
       <c r="B26">
-        <v>8.75</v>
+        <v>5.75</v>
       </c>
       <c r="C26">
-        <v>9.75</v>
+        <v>8.5</v>
       </c>
       <c r="D26">
-        <v>14.75</v>
+        <v>13.5</v>
       </c>
       <c r="E26">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G26">
-        <v>9.050000000000001</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -6855,22 +6855,22 @@
         <v>33</v>
       </c>
       <c r="B28">
-        <v>6.5</v>
+        <v>4.25</v>
       </c>
       <c r="C28">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D28">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E28">
-        <v>8.75</v>
+        <v>6.75</v>
       </c>
       <c r="F28">
         <v>2</v>
       </c>
       <c r="G28">
-        <v>7.65</v>
+        <v>6.15</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -6878,22 +6878,22 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>6.75</v>
+        <v>4.5</v>
       </c>
       <c r="C29">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="D29">
-        <v>13.75</v>
+        <v>12.25</v>
       </c>
       <c r="E29">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="F29">
         <v>4</v>
       </c>
       <c r="G29">
-        <v>8.15</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -6901,22 +6901,22 @@
         <v>35</v>
       </c>
       <c r="B30">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C30">
-        <v>8.5</v>
+        <v>7</v>
       </c>
       <c r="D30">
-        <v>14.5</v>
+        <v>12.75</v>
       </c>
       <c r="E30">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="F30">
-        <v>5.25</v>
+        <v>4.25</v>
       </c>
       <c r="G30">
-        <v>8.699999999999999</v>
+        <v>6.95</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -6947,22 +6947,22 @@
         <v>37</v>
       </c>
       <c r="B32">
-        <v>8.25</v>
+        <v>5.5</v>
       </c>
       <c r="C32">
-        <v>8.5</v>
+        <v>7.25</v>
       </c>
       <c r="D32">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E32">
-        <v>9.25</v>
+        <v>6.5</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32">
-        <v>8.199999999999999</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -7016,22 +7016,22 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C35">
-        <v>9</v>
+        <v>5.75</v>
       </c>
       <c r="D35">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E35">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F35">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="G35">
-        <v>7.6</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -7039,22 +7039,22 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>6</v>
+        <v>4.25</v>
       </c>
       <c r="C36">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="D36">
-        <v>13.5</v>
+        <v>12.25</v>
       </c>
       <c r="E36">
-        <v>8.25</v>
+        <v>4.75</v>
       </c>
       <c r="F36">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>8.6</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -7085,22 +7085,22 @@
         <v>43</v>
       </c>
       <c r="B38">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C38">
-        <v>8.5</v>
+        <v>6.25</v>
       </c>
       <c r="D38">
-        <v>13</v>
+        <v>12.25</v>
       </c>
       <c r="E38">
-        <v>9.25</v>
+        <v>6.75</v>
       </c>
       <c r="F38">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="G38">
-        <v>7.75</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -7108,22 +7108,22 @@
         <v>44</v>
       </c>
       <c r="B39">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="C39">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="D39">
-        <v>13.75</v>
+        <v>12.25</v>
       </c>
       <c r="E39">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F39">
         <v>4</v>
       </c>
       <c r="G39">
-        <v>8.15</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -7131,22 +7131,22 @@
         <v>45</v>
       </c>
       <c r="B40">
-        <v>8.75</v>
+        <v>5</v>
       </c>
       <c r="C40">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D40">
-        <v>14.5</v>
+        <v>12.75</v>
       </c>
       <c r="E40">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F40">
-        <v>5.25</v>
+        <v>4.25</v>
       </c>
       <c r="G40">
-        <v>8.9</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -7177,22 +7177,22 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>9</v>
+        <v>6.25</v>
       </c>
       <c r="C42">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="D42">
-        <v>14.75</v>
+        <v>13.5</v>
       </c>
       <c r="E42">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G42">
-        <v>9.050000000000001</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -7200,22 +7200,22 @@
         <v>48</v>
       </c>
       <c r="B43">
+        <v>4.5</v>
+      </c>
+      <c r="C43">
         <v>7</v>
       </c>
-      <c r="C43">
-        <v>8.5</v>
-      </c>
       <c r="D43">
-        <v>14.75</v>
+        <v>12.75</v>
       </c>
       <c r="E43">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F43">
-        <v>4.75</v>
+        <v>4.25</v>
       </c>
       <c r="G43">
-        <v>8.4</v>
+        <v>6.85</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -7223,22 +7223,22 @@
         <v>49</v>
       </c>
       <c r="B44">
+        <v>4.75</v>
+      </c>
+      <c r="C44">
         <v>6.75</v>
       </c>
-      <c r="C44">
-        <v>9.75</v>
-      </c>
       <c r="D44">
-        <v>13</v>
+        <v>10.75</v>
       </c>
       <c r="E44">
-        <v>9.25</v>
+        <v>6.5</v>
       </c>
       <c r="F44">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="G44">
-        <v>8.6</v>
+        <v>6.55</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -7269,22 +7269,22 @@
         <v>51</v>
       </c>
       <c r="B46">
+        <v>5</v>
+      </c>
+      <c r="C46">
         <v>7</v>
       </c>
-      <c r="C46">
-        <v>10</v>
-      </c>
       <c r="D46">
-        <v>14</v>
+        <v>12.5</v>
       </c>
       <c r="E46">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F46">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="G46">
-        <v>8.550000000000001</v>
+        <v>6.85</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -7292,22 +7292,22 @@
         <v>52</v>
       </c>
       <c r="B47">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C47">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="D47">
-        <v>14.5</v>
+        <v>13.25</v>
       </c>
       <c r="E47">
-        <v>7.75</v>
+        <v>6.5</v>
       </c>
       <c r="F47">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="G47">
-        <v>8.6</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -7315,22 +7315,22 @@
         <v>53</v>
       </c>
       <c r="B48">
+        <v>4.5</v>
+      </c>
+      <c r="C48">
         <v>7.5</v>
       </c>
-      <c r="C48">
-        <v>9</v>
-      </c>
       <c r="D48">
-        <v>14.75</v>
+        <v>12.75</v>
       </c>
       <c r="E48">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="F48">
-        <v>4.75</v>
+        <v>4.25</v>
       </c>
       <c r="G48">
-        <v>8.6</v>
+        <v>6.95</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -7338,22 +7338,22 @@
         <v>54</v>
       </c>
       <c r="B49">
+        <v>5</v>
+      </c>
+      <c r="C49">
         <v>7</v>
       </c>
-      <c r="C49">
-        <v>10</v>
-      </c>
       <c r="D49">
-        <v>14</v>
+        <v>12.5</v>
       </c>
       <c r="E49">
-        <v>7.75</v>
+        <v>6.25</v>
       </c>
       <c r="F49">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="G49">
-        <v>8.699999999999999</v>
+        <v>6.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>